<commit_message>
Isca xlsx: CC-01 faixa seguro-desemprego, SM diário/horário, INSS faixa cheia como derivado
</commit_message>
<xml_diff>
--- a/tabelas-oficiais-2026/tabelas-oficiais-2026-conta-certa.xlsx
+++ b/tabelas-oficiais-2026/tabelas-oficiais-2026-conta-certa.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Contribuição da faixa cheia (R$)</t>
+          <t>Contribuição da faixa cheia (R$) - valor derivado (calculado pelo Conta Certa)</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -861,59 +861,79 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vigência</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>01/01/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+          <t>Salário mínimo diário (R$) - derivado: mensal / 30</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>54.03</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Salário mínimo por hora (R$) - derivado: mensal / 220</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.37</v>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fonte oficial:</t>
+          <t>Vigência</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Decreto nº 12.797, de 23/12/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Link:</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.planalto.gov.br/ccivil_03/_ato2023-2026/2025/decreto/d12797.htm</t>
-        </is>
-      </c>
-    </row>
+          <t>01/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Conferido em:</t>
+          <t>Fonte oficial:</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>Decreto nº 12.797, de 23/12/2025</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Link:</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.planalto.gov.br/ccivil_03/_ato2023-2026/2025/decreto/d12797.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Conferido em:</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Aviso:</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Consulta; não substitui a fonte oficial nem orientação profissional. contacertabr.com.br</t>
         </is>
@@ -973,7 +993,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>De R$ 2.222,17 a R$ 3.703,99</t>
+          <t>De R$ 2.222,18 a R$ 3.703,99</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>

<commit_message>
Isca xlsx: salário mínimo diário R$ 54,04 e horário R$ 7,37 pelo Decreto 12.797/2025, art. 1º, p. único
</commit_message>
<xml_diff>
--- a/tabelas-oficiais-2026/tabelas-oficiais-2026-conta-certa.xlsx
+++ b/tabelas-oficiais-2026/tabelas-oficiais-2026-conta-certa.xlsx
@@ -861,17 +861,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Salário mínimo diário (R$) - derivado: mensal / 30</t>
+          <t>Salário mínimo diário (R$) - Decreto nº 12.797/2025, art. 1º, parágrafo único</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>54.03</v>
+        <v>54.04</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Salário mínimo por hora (R$) - derivado: mensal / 220</t>
+          <t>Salário mínimo horário (R$) - Decreto nº 12.797/2025, art. 1º, parágrafo único</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">

</xml_diff>